<commit_message>
Implement incremental sofascore scraping pipeline
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/Server/files_initted/partidos_info.xlsx
+++ b/webscrapping/sofascore/Server/files_initted/partidos_info.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="152">
   <si>
     <t>Jornada</t>
   </si>
@@ -211,6 +211,36 @@
     <t>01/12/2025</t>
   </si>
   <si>
+    <t>05/12/2025</t>
+  </si>
+  <si>
+    <t>06/12/2025</t>
+  </si>
+  <si>
+    <t>07/12/2025</t>
+  </si>
+  <si>
+    <t>08/12/2025</t>
+  </si>
+  <si>
+    <t>12/12/2025</t>
+  </si>
+  <si>
+    <t>13/12/2025</t>
+  </si>
+  <si>
+    <t>14/12/2025</t>
+  </si>
+  <si>
+    <t>15/12/2025</t>
+  </si>
+  <si>
+    <t>19/12/2025</t>
+  </si>
+  <si>
+    <t>20/12/2025</t>
+  </si>
+  <si>
     <t>19:00</t>
   </si>
   <si>
@@ -368,6 +398,9 @@
   </si>
   <si>
     <t>2-4</t>
+  </si>
+  <si>
+    <t>3-5</t>
   </si>
   <si>
     <t>Estadi Montilivi</t>
@@ -794,7 +827,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -849,19 +882,19 @@
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H2" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="I2" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J2">
         <v>14624</v>
@@ -887,19 +920,19 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H3" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I3" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J3">
         <v>23500</v>
@@ -925,19 +958,19 @@
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G4" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H4" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="I4" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J4">
         <v>26020</v>
@@ -963,19 +996,19 @@
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H5" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I5" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J5">
         <v>19840</v>
@@ -1001,19 +1034,19 @@
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G6" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H6" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I6" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J6">
         <v>49430</v>
@@ -1039,19 +1072,19 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H7" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J7">
         <v>24870</v>
@@ -1077,19 +1110,19 @@
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G8" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H8" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I8" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J8">
         <v>53289</v>
@@ -1115,19 +1148,19 @@
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G9" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H9" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I9" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J9">
         <v>40000</v>
@@ -1153,19 +1186,19 @@
         <v>15</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G10" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H10" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J10">
         <v>31388</v>
@@ -1191,19 +1224,19 @@
         <v>16</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G11" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H11" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I11" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="J11">
         <v>84744</v>
@@ -1229,19 +1262,19 @@
         <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F12" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G12" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H12" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I12" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="J12">
         <v>60721</v>
@@ -1267,19 +1300,19 @@
         <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G13" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H13" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I13" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J13">
         <v>26020</v>
@@ -1305,19 +1338,19 @@
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F14" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G14" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H14" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I14" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J14">
         <v>70460</v>
@@ -1343,19 +1376,19 @@
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H15" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I15" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J15">
         <v>26354</v>
@@ -1381,19 +1414,19 @@
         <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F16" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G16" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I16" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J16">
         <v>23576</v>
@@ -1419,19 +1452,19 @@
         <v>19</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G17" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H17" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I17" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J17">
         <v>40000</v>
@@ -1457,19 +1490,19 @@
         <v>19</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F18" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G18" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H18" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I18" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J18">
         <v>23500</v>
@@ -1495,19 +1528,19 @@
         <v>19</v>
       </c>
       <c r="E19" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G19" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H19" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="I19" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J19">
         <v>30500</v>
@@ -1533,19 +1566,19 @@
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F20" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G20" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H20" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I20" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J20">
         <v>53289</v>
@@ -1571,19 +1604,19 @@
         <v>20</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F21" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G21" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H21" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I21" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J21">
         <v>42714</v>
@@ -1609,19 +1642,19 @@
         <v>21</v>
       </c>
       <c r="E22" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F22" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G22" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H22" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I22" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J22">
         <v>31388</v>
@@ -1647,19 +1680,19 @@
         <v>21</v>
       </c>
       <c r="E23" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F23" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G23" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H23" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I23" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J23">
         <v>49430</v>
@@ -1685,19 +1718,19 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F24" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G24" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H24" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I24" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J24">
         <v>19840</v>
@@ -1723,19 +1756,19 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F25" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G25" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H25" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I25" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J25">
         <v>30500</v>
@@ -1761,19 +1794,19 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F26" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G26" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H26" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I26" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J26">
         <v>14624</v>
@@ -1799,19 +1832,19 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F27" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G27" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H27" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I27" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="J27">
         <v>84744</v>
@@ -1837,19 +1870,19 @@
         <v>23</v>
       </c>
       <c r="E28" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F28" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G28" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H28" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I28" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J28">
         <v>24870</v>
@@ -1875,19 +1908,19 @@
         <v>23</v>
       </c>
       <c r="E29" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F29" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G29" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H29" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I29" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="J29">
         <v>60721</v>
@@ -1913,19 +1946,19 @@
         <v>23</v>
       </c>
       <c r="E30" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F30" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G30" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H30" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I30" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J30">
         <v>40000</v>
@@ -1951,19 +1984,19 @@
         <v>23</v>
       </c>
       <c r="E31" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F31" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G31" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H31" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I31" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J31">
         <v>14708</v>
@@ -1989,19 +2022,19 @@
         <v>24</v>
       </c>
       <c r="E32" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F32" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G32" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H32" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I32" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J32">
         <v>42714</v>
@@ -2027,19 +2060,19 @@
         <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F33" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G33" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H33" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I33" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J33">
         <v>17393</v>
@@ -2065,19 +2098,19 @@
         <v>25</v>
       </c>
       <c r="E34" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F34" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G34" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H34" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I34" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J34">
         <v>40000</v>
@@ -2103,19 +2136,19 @@
         <v>25</v>
       </c>
       <c r="E35" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F35" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G35" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H35" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I35" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J35">
         <v>53289</v>
@@ -2141,19 +2174,19 @@
         <v>25</v>
       </c>
       <c r="E36" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F36" t="s">
+        <v>95</v>
+      </c>
+      <c r="G36" t="s">
         <v>85</v>
       </c>
-      <c r="G36" t="s">
-        <v>75</v>
-      </c>
       <c r="H36" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I36" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J36">
         <v>70460</v>
@@ -2179,19 +2212,19 @@
         <v>26</v>
       </c>
       <c r="E37" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F37" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G37" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H37" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I37" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J37">
         <v>24870</v>
@@ -2217,19 +2250,19 @@
         <v>26</v>
       </c>
       <c r="E38" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F38" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G38" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H38" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I38" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J38">
         <v>26354</v>
@@ -2255,19 +2288,19 @@
         <v>26</v>
       </c>
       <c r="E39" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G39" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H39" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I39" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J39">
         <v>23576</v>
@@ -2293,19 +2326,19 @@
         <v>26</v>
       </c>
       <c r="E40" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F40" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G40" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H40" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="I40" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="J40">
         <v>6000</v>
@@ -2331,19 +2364,19 @@
         <v>27</v>
       </c>
       <c r="E41" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F41" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G41" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H41" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I41" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J41">
         <v>40000</v>
@@ -2369,19 +2402,19 @@
         <v>28</v>
       </c>
       <c r="E42" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F42" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G42" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H42" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I42" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="J42">
         <v>60721</v>
@@ -2407,19 +2440,19 @@
         <v>29</v>
       </c>
       <c r="E43" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F43" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G43" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H43" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="I43" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J43">
         <v>14624</v>
@@ -2445,19 +2478,19 @@
         <v>29</v>
       </c>
       <c r="E44" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F44" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G44" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H44" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I44" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="J44">
         <v>84744</v>
@@ -2483,19 +2516,19 @@
         <v>29</v>
       </c>
       <c r="E45" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F45" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G45" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H45" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I45" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J45">
         <v>19840</v>
@@ -2521,19 +2554,19 @@
         <v>29</v>
       </c>
       <c r="E46" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F46" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G46" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H46" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I46" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J46">
         <v>23500</v>
@@ -2559,19 +2592,19 @@
         <v>29</v>
       </c>
       <c r="E47" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F47" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G47" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H47" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I47" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J47">
         <v>49430</v>
@@ -2597,19 +2630,19 @@
         <v>30</v>
       </c>
       <c r="E48" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F48" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G48" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H48" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I48" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J48">
         <v>14708</v>
@@ -2635,19 +2668,19 @@
         <v>30</v>
       </c>
       <c r="E49" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F49" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G49" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H49" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I49" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J49">
         <v>26020</v>
@@ -2673,19 +2706,19 @@
         <v>30</v>
       </c>
       <c r="E50" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F50" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G50" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H50" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I50" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J50">
         <v>31388</v>
@@ -2711,19 +2744,19 @@
         <v>30</v>
       </c>
       <c r="E51" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F51" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G51" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H51" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I51" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="J51">
         <v>6000</v>
@@ -2749,19 +2782,19 @@
         <v>31</v>
       </c>
       <c r="E52" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F52" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G52" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H52" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I52" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J52">
         <v>24870</v>
@@ -2787,19 +2820,19 @@
         <v>32</v>
       </c>
       <c r="E53" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F53" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G53" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H53" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I53" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J53">
         <v>53289</v>
@@ -2825,19 +2858,19 @@
         <v>32</v>
       </c>
       <c r="E54" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F54" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G54" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H54" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I54" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J54">
         <v>40000</v>
@@ -2863,19 +2896,19 @@
         <v>32</v>
       </c>
       <c r="E55" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F55" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G55" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H55" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="I55" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J55">
         <v>26354</v>
@@ -2901,19 +2934,19 @@
         <v>32</v>
       </c>
       <c r="E56" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F56" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G56" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H56" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I56" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J56">
         <v>42714</v>
@@ -2939,19 +2972,19 @@
         <v>33</v>
       </c>
       <c r="E57" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F57" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G57" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H57" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I57" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J57">
         <v>17393</v>
@@ -2977,19 +3010,19 @@
         <v>33</v>
       </c>
       <c r="E58" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F58" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G58" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H58" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I58" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J58">
         <v>70460</v>
@@ -3015,19 +3048,19 @@
         <v>33</v>
       </c>
       <c r="E59" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F59" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G59" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H59" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I59" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J59">
         <v>40000</v>
@@ -3053,19 +3086,19 @@
         <v>34</v>
       </c>
       <c r="E60" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F60" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G60" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H60" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I60" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J60">
         <v>23576</v>
@@ -3091,19 +3124,19 @@
         <v>34</v>
       </c>
       <c r="E61" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F61" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G61" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H61" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="I61" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J61">
         <v>30500</v>
@@ -3129,19 +3162,19 @@
         <v>35</v>
       </c>
       <c r="E62" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F62" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G62" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H62" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I62" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J62">
         <v>14624</v>
@@ -3167,19 +3200,19 @@
         <v>36</v>
       </c>
       <c r="E63" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F63" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G63" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H63" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I63" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J63">
         <v>17393</v>
@@ -3205,19 +3238,19 @@
         <v>36</v>
       </c>
       <c r="E64" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F64" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G64" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H64" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="I64" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J64">
         <v>70460</v>
@@ -3243,19 +3276,19 @@
         <v>36</v>
       </c>
       <c r="E65" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F65" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G65" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H65" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I65" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J65">
         <v>26020</v>
@@ -3281,19 +3314,19 @@
         <v>36</v>
       </c>
       <c r="E66" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F66" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G66" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H66" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I66" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J66">
         <v>23500</v>
@@ -3319,19 +3352,19 @@
         <v>37</v>
       </c>
       <c r="E67" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F67" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G67" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H67" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I67" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J67">
         <v>14708</v>
@@ -3357,19 +3390,19 @@
         <v>37</v>
       </c>
       <c r="E68" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F68" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G68" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H68" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I68" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J68">
         <v>31388</v>
@@ -3395,19 +3428,19 @@
         <v>37</v>
       </c>
       <c r="E69" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F69" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G69" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H69" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I69" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="J69">
         <v>55926</v>
@@ -3433,19 +3466,19 @@
         <v>37</v>
       </c>
       <c r="E70" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F70" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G70" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H70" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I70" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="J70">
         <v>70000</v>
@@ -3471,19 +3504,19 @@
         <v>38</v>
       </c>
       <c r="E71" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="F71" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G71" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H71" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I71" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J71">
         <v>49430</v>
@@ -3509,19 +3542,19 @@
         <v>39</v>
       </c>
       <c r="E72" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F72" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G72" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H72" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I72" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J72">
         <v>23576</v>
@@ -3547,19 +3580,19 @@
         <v>40</v>
       </c>
       <c r="E73" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F73" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G73" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H73" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I73" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J73">
         <v>30500</v>
@@ -3585,19 +3618,19 @@
         <v>40</v>
       </c>
       <c r="E74" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F74" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G74" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H74" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I74" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J74">
         <v>14624</v>
@@ -3623,19 +3656,19 @@
         <v>40</v>
       </c>
       <c r="E75" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F75" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G75" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H75" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I75" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J75">
         <v>53289</v>
@@ -3661,19 +3694,19 @@
         <v>40</v>
       </c>
       <c r="E76" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F76" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G76" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H76" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I76" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="J76">
         <v>84744</v>
@@ -3699,19 +3732,19 @@
         <v>41</v>
       </c>
       <c r="E77" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F77" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G77" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H77" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I77" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J77">
         <v>19840</v>
@@ -3737,19 +3770,19 @@
         <v>41</v>
       </c>
       <c r="E78" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F78" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G78" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H78" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="I78" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J78">
         <v>42714</v>
@@ -3775,19 +3808,19 @@
         <v>41</v>
       </c>
       <c r="E79" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F79" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G79" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H79" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I79" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J79">
         <v>40000</v>
@@ -3813,19 +3846,19 @@
         <v>41</v>
       </c>
       <c r="E80" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F80" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G80" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H80" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I80" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J80">
         <v>40000</v>
@@ -3851,19 +3884,19 @@
         <v>41</v>
       </c>
       <c r="E81" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F81" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G81" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H81" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I81" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J81">
         <v>24870</v>
@@ -3889,19 +3922,19 @@
         <v>42</v>
       </c>
       <c r="E82" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F82" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G82" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H82" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I82" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J82">
         <v>30500</v>
@@ -3927,19 +3960,19 @@
         <v>43</v>
       </c>
       <c r="E83" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F83" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G83" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H83" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="I83" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J83">
         <v>42714</v>
@@ -3965,19 +3998,19 @@
         <v>43</v>
       </c>
       <c r="E84" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F84" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G84" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H84" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I84" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="J84">
         <v>55926</v>
@@ -4003,19 +4036,19 @@
         <v>43</v>
       </c>
       <c r="E85" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F85" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G85" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H85" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I85" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J85">
         <v>23500</v>
@@ -4041,19 +4074,19 @@
         <v>43</v>
       </c>
       <c r="E86" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F86" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G86" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H86" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I86" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J86">
         <v>70460</v>
@@ -4079,19 +4112,19 @@
         <v>44</v>
       </c>
       <c r="E87" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F87" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G87" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H87" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I87" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J87">
         <v>31388</v>
@@ -4117,19 +4150,19 @@
         <v>44</v>
       </c>
       <c r="E88" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F88" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G88" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H88" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I88" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J88">
         <v>24870</v>
@@ -4155,19 +4188,19 @@
         <v>44</v>
       </c>
       <c r="E89" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F89" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G89" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H89" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="I89" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J89">
         <v>26354</v>
@@ -4193,19 +4226,19 @@
         <v>44</v>
       </c>
       <c r="E90" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F90" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G90" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H90" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I90" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J90">
         <v>17393</v>
@@ -4231,19 +4264,19 @@
         <v>45</v>
       </c>
       <c r="E91" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F91" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G91" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H91" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I91" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J91">
         <v>19840</v>
@@ -4269,19 +4302,19 @@
         <v>46</v>
       </c>
       <c r="E92" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F92" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G92" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H92" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I92" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J92">
         <v>40000</v>
@@ -4307,19 +4340,19 @@
         <v>47</v>
       </c>
       <c r="E93" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F93" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G93" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H93" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="I93" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J93">
         <v>14624</v>
@@ -4345,19 +4378,19 @@
         <v>47</v>
       </c>
       <c r="E94" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F94" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G94" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H94" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I94" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J94">
         <v>40000</v>
@@ -4383,19 +4416,19 @@
         <v>47</v>
       </c>
       <c r="E95" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F95" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G95" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H95" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I95" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J95">
         <v>53289</v>
@@ -4421,19 +4454,19 @@
         <v>47</v>
       </c>
       <c r="E96" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F96" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G96" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H96" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I96" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J96">
         <v>49430</v>
@@ -4459,19 +4492,19 @@
         <v>48</v>
       </c>
       <c r="E97" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F97" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G97" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H97" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I97" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J97">
         <v>26020</v>
@@ -4497,19 +4530,19 @@
         <v>48</v>
       </c>
       <c r="E98" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F98" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G98" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H98" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I98" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="J98">
         <v>84744</v>
@@ -4535,19 +4568,19 @@
         <v>48</v>
       </c>
       <c r="E99" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F99" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G99" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H99" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I99" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J99">
         <v>23576</v>
@@ -4573,19 +4606,19 @@
         <v>48</v>
       </c>
       <c r="E100" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F100" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G100" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H100" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I100" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J100">
         <v>14708</v>
@@ -4611,19 +4644,19 @@
         <v>49</v>
       </c>
       <c r="E101" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F101" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G101" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H101" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I101" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="J101">
         <v>70000</v>
@@ -4649,19 +4682,19 @@
         <v>50</v>
       </c>
       <c r="E102" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F102" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G102" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H102" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I102" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J102">
         <v>17393</v>
@@ -4687,19 +4720,19 @@
         <v>51</v>
       </c>
       <c r="E103" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F103" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G103" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H103" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="I103" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J103">
         <v>23500</v>
@@ -4725,19 +4758,19 @@
         <v>51</v>
       </c>
       <c r="E104" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F104" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G104" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H104" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I104" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J104">
         <v>70460</v>
@@ -4763,19 +4796,19 @@
         <v>51</v>
       </c>
       <c r="E105" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F105" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G105" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H105" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I105" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J105">
         <v>40000</v>
@@ -4801,19 +4834,19 @@
         <v>51</v>
       </c>
       <c r="E106" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F106" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G106" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H106" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="I106" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="J106">
         <v>84744</v>
@@ -4839,19 +4872,19 @@
         <v>52</v>
       </c>
       <c r="E107" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F107" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G107" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H107" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="I107" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J107">
         <v>26354</v>
@@ -4877,19 +4910,19 @@
         <v>52</v>
       </c>
       <c r="E108" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F108" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G108" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H108" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I108" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J108">
         <v>19840</v>
@@ -4915,19 +4948,19 @@
         <v>52</v>
       </c>
       <c r="E109" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F109" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G109" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H109" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I109" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="J109">
         <v>55926</v>
@@ -4953,19 +4986,19 @@
         <v>52</v>
       </c>
       <c r="E110" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F110" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G110" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H110" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I110" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="J110">
         <v>60721</v>
@@ -4991,19 +5024,19 @@
         <v>53</v>
       </c>
       <c r="E111" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F111" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G111" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H111" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I111" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J111">
         <v>30500</v>
@@ -5029,19 +5062,19 @@
         <v>54</v>
       </c>
       <c r="E112" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F112" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G112" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H112" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I112" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J112">
         <v>31388</v>
@@ -5067,19 +5100,19 @@
         <v>55</v>
       </c>
       <c r="E113" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F113" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G113" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H113" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I113" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J113">
         <v>14624</v>
@@ -5105,19 +5138,19 @@
         <v>55</v>
       </c>
       <c r="E114" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F114" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G114" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H114" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I114" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J114">
         <v>42714</v>
@@ -5143,19 +5176,19 @@
         <v>55</v>
       </c>
       <c r="E115" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F115" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G115" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H115" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I115" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J115">
         <v>70460</v>
@@ -5181,19 +5214,19 @@
         <v>55</v>
       </c>
       <c r="E116" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F116" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G116" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H116" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I116" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J116">
         <v>40000</v>
@@ -5219,19 +5252,19 @@
         <v>56</v>
       </c>
       <c r="E117" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F117" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G117" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H117" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I117" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J117">
         <v>53289</v>
@@ -5257,19 +5290,19 @@
         <v>56</v>
       </c>
       <c r="E118" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F118" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G118" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H118" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I118" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J118">
         <v>14708</v>
@@ -5295,19 +5328,19 @@
         <v>56</v>
       </c>
       <c r="E119" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F119" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G119" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="H119" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I119" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J119">
         <v>26020</v>
@@ -5333,19 +5366,19 @@
         <v>56</v>
       </c>
       <c r="E120" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F120" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G120" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H120" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I120" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J120">
         <v>49430</v>
@@ -5371,19 +5404,19 @@
         <v>56</v>
       </c>
       <c r="E121" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F121" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G121" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H121" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="I121" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J121">
         <v>24870</v>
@@ -5409,19 +5442,19 @@
         <v>57</v>
       </c>
       <c r="E122" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F122" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G122" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H122" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I122" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J122">
         <v>49430</v>
@@ -5447,19 +5480,19 @@
         <v>58</v>
       </c>
       <c r="E123" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F123" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G123" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H123" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I123" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J123">
         <v>19840</v>
@@ -5485,19 +5518,19 @@
         <v>58</v>
       </c>
       <c r="E124" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F124" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G124" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H124" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="I124" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="J124">
         <v>45401</v>
@@ -5523,19 +5556,19 @@
         <v>58</v>
       </c>
       <c r="E125" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F125" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G125" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H125" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="I125" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="J125">
         <v>23576</v>
@@ -5561,19 +5594,19 @@
         <v>58</v>
       </c>
       <c r="E126" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F126" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G126" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H126" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I126" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J126">
         <v>23500</v>
@@ -5599,19 +5632,19 @@
         <v>59</v>
       </c>
       <c r="E127" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F127" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G127" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="H127" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="I127" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="J127">
         <v>30500</v>
@@ -5637,19 +5670,19 @@
         <v>59</v>
       </c>
       <c r="E128" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F128" t="s">
+        <v>94</v>
+      </c>
+      <c r="G128" t="s">
         <v>84</v>
       </c>
-      <c r="G128" t="s">
-        <v>74</v>
-      </c>
       <c r="H128" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I128" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="J128">
         <v>70000</v>
@@ -5675,19 +5708,19 @@
         <v>59</v>
       </c>
       <c r="E129" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F129" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G129" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H129" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I129" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J129">
         <v>17393</v>
@@ -5713,19 +5746,19 @@
         <v>59</v>
       </c>
       <c r="E130" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F130" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="G130" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H130" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I130" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="J130">
         <v>31388</v>
@@ -5751,19 +5784,19 @@
         <v>60</v>
       </c>
       <c r="E131" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F131" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G131" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H131" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I131" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="J131">
         <v>40000</v>
@@ -5789,19 +5822,19 @@
         <v>61</v>
       </c>
       <c r="E132" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F132" t="s">
+        <v>102</v>
+      </c>
+      <c r="G132" t="s">
         <v>92</v>
       </c>
-      <c r="G132" t="s">
-        <v>82</v>
-      </c>
       <c r="H132" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I132" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="J132">
         <v>17393</v>
@@ -5827,19 +5860,19 @@
         <v>62</v>
       </c>
       <c r="E133" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F133" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G133" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="H133" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="I133" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J133">
         <v>26020</v>
@@ -5865,19 +5898,19 @@
         <v>62</v>
       </c>
       <c r="E134" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F134" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G134" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H134" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="I134" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="J134">
         <v>45401</v>
@@ -5903,19 +5936,19 @@
         <v>62</v>
       </c>
       <c r="E135" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F135" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G135" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H135" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I135" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J135">
         <v>26354</v>
@@ -5941,19 +5974,19 @@
         <v>62</v>
       </c>
       <c r="E136" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F136" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G136" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H136" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I136" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J136">
         <v>70460</v>
@@ -5979,19 +6012,19 @@
         <v>63</v>
       </c>
       <c r="E137" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F137" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G137" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H137" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="I137" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J137">
         <v>40000</v>
@@ -6017,19 +6050,19 @@
         <v>63</v>
       </c>
       <c r="E138" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F138" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G138" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H138" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I138" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J138">
         <v>42714</v>
@@ -6055,19 +6088,19 @@
         <v>63</v>
       </c>
       <c r="E139" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F139" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G139" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H139" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I139" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="J139">
         <v>24870</v>
@@ -6093,19 +6126,19 @@
         <v>63</v>
       </c>
       <c r="E140" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F140" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="G140" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H140" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I140" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J140">
         <v>14624</v>
@@ -6131,19 +6164,19 @@
         <v>64</v>
       </c>
       <c r="E141" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F141" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G141" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H141" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I141" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="J141">
         <v>14708</v>
@@ -6153,6 +6186,918 @@
       </c>
       <c r="L141">
         <v>-3.6587</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12">
+      <c r="A142">
+        <v>15</v>
+      </c>
+      <c r="B142">
+        <v>1</v>
+      </c>
+      <c r="C142">
+        <v>14083162</v>
+      </c>
+      <c r="D142" t="s">
+        <v>65</v>
+      </c>
+      <c r="E142" t="s">
+        <v>79</v>
+      </c>
+      <c r="F142" t="s">
+        <v>99</v>
+      </c>
+      <c r="G142" t="s">
+        <v>86</v>
+      </c>
+      <c r="H142" t="s">
+        <v>122</v>
+      </c>
+      <c r="I142" t="s">
+        <v>144</v>
+      </c>
+      <c r="J142">
+        <v>30500</v>
+      </c>
+      <c r="K142">
+        <v>43.360872</v>
+      </c>
+      <c r="L142">
+        <v>-5.870332</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12">
+      <c r="A143">
+        <v>15</v>
+      </c>
+      <c r="B143">
+        <v>2</v>
+      </c>
+      <c r="C143">
+        <v>14083159</v>
+      </c>
+      <c r="D143" t="s">
+        <v>66</v>
+      </c>
+      <c r="E143" t="s">
+        <v>80</v>
+      </c>
+      <c r="F143" t="s">
+        <v>85</v>
+      </c>
+      <c r="G143" t="s">
+        <v>102</v>
+      </c>
+      <c r="H143" t="s">
+        <v>105</v>
+      </c>
+      <c r="I143" t="s">
+        <v>130</v>
+      </c>
+      <c r="J143">
+        <v>23500</v>
+      </c>
+      <c r="K143">
+        <v>39.944208</v>
+      </c>
+      <c r="L143">
+        <v>-0.103405</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12">
+      <c r="A144">
+        <v>15</v>
+      </c>
+      <c r="B144">
+        <v>3</v>
+      </c>
+      <c r="C144">
+        <v>14083150</v>
+      </c>
+      <c r="D144" t="s">
+        <v>66</v>
+      </c>
+      <c r="E144" t="s">
+        <v>81</v>
+      </c>
+      <c r="F144" t="s">
+        <v>87</v>
+      </c>
+      <c r="G144" t="s">
+        <v>98</v>
+      </c>
+      <c r="H144" t="s">
+        <v>111</v>
+      </c>
+      <c r="I144" t="s">
+        <v>132</v>
+      </c>
+      <c r="J144">
+        <v>19840</v>
+      </c>
+      <c r="K144">
+        <v>42.8371</v>
+      </c>
+      <c r="L144">
+        <v>-2.6882</v>
+      </c>
+    </row>
+    <row r="145" spans="1:12">
+      <c r="A145">
+        <v>15</v>
+      </c>
+      <c r="B145">
+        <v>4</v>
+      </c>
+      <c r="C145">
+        <v>14083155</v>
+      </c>
+      <c r="D145" t="s">
+        <v>66</v>
+      </c>
+      <c r="E145" t="s">
+        <v>82</v>
+      </c>
+      <c r="F145" t="s">
+        <v>94</v>
+      </c>
+      <c r="G145" t="s">
+        <v>103</v>
+      </c>
+      <c r="H145" t="s">
+        <v>128</v>
+      </c>
+      <c r="I145" t="s">
+        <v>150</v>
+      </c>
+      <c r="J145">
+        <v>70000</v>
+      </c>
+      <c r="K145">
+        <v>37.417235</v>
+      </c>
+      <c r="L145">
+        <v>-6.004613</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12">
+      <c r="A146">
+        <v>15</v>
+      </c>
+      <c r="B146">
+        <v>5</v>
+      </c>
+      <c r="C146">
+        <v>14083151</v>
+      </c>
+      <c r="D146" t="s">
+        <v>66</v>
+      </c>
+      <c r="E146" t="s">
+        <v>79</v>
+      </c>
+      <c r="F146" t="s">
+        <v>90</v>
+      </c>
+      <c r="G146" t="s">
+        <v>95</v>
+      </c>
+      <c r="H146" t="s">
+        <v>111</v>
+      </c>
+      <c r="I146" t="s">
+        <v>135</v>
+      </c>
+      <c r="J146">
+        <v>53289</v>
+      </c>
+      <c r="K146">
+        <v>43.264204</v>
+      </c>
+      <c r="L146">
+        <v>-2.949391</v>
+      </c>
+    </row>
+    <row r="147" spans="1:12">
+      <c r="A147">
+        <v>15</v>
+      </c>
+      <c r="B147">
+        <v>6</v>
+      </c>
+      <c r="C147">
+        <v>14083153</v>
+      </c>
+      <c r="D147" t="s">
+        <v>67</v>
+      </c>
+      <c r="E147" t="s">
+        <v>80</v>
+      </c>
+      <c r="F147" t="s">
+        <v>92</v>
+      </c>
+      <c r="G147" t="s">
+        <v>84</v>
+      </c>
+      <c r="H147" t="s">
+        <v>116</v>
+      </c>
+      <c r="I147" t="s">
+        <v>137</v>
+      </c>
+      <c r="J147">
+        <v>31388</v>
+      </c>
+      <c r="K147">
+        <v>38.267044</v>
+      </c>
+      <c r="L147">
+        <v>-0.663305</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12">
+      <c r="A148">
+        <v>15</v>
+      </c>
+      <c r="B148">
+        <v>7</v>
+      </c>
+      <c r="C148">
+        <v>14083163</v>
+      </c>
+      <c r="D148" t="s">
+        <v>67</v>
+      </c>
+      <c r="E148" t="s">
+        <v>81</v>
+      </c>
+      <c r="F148" t="s">
+        <v>88</v>
+      </c>
+      <c r="G148" t="s">
+        <v>100</v>
+      </c>
+      <c r="H148" t="s">
+        <v>108</v>
+      </c>
+      <c r="I148" t="s">
+        <v>133</v>
+      </c>
+      <c r="J148">
+        <v>49430</v>
+      </c>
+      <c r="K148">
+        <v>39.474528</v>
+      </c>
+      <c r="L148">
+        <v>-0.358157</v>
+      </c>
+    </row>
+    <row r="149" spans="1:12">
+      <c r="A149">
+        <v>15</v>
+      </c>
+      <c r="B149">
+        <v>8</v>
+      </c>
+      <c r="C149">
+        <v>14083154</v>
+      </c>
+      <c r="D149" t="s">
+        <v>67</v>
+      </c>
+      <c r="E149" t="s">
+        <v>82</v>
+      </c>
+      <c r="F149" t="s">
+        <v>91</v>
+      </c>
+      <c r="G149" t="s">
+        <v>101</v>
+      </c>
+      <c r="H149" t="s">
+        <v>111</v>
+      </c>
+      <c r="I149" t="s">
+        <v>136</v>
+      </c>
+      <c r="J149">
+        <v>40000</v>
+      </c>
+      <c r="K149">
+        <v>41.347807</v>
+      </c>
+      <c r="L149">
+        <v>2.074801</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12">
+      <c r="A150">
+        <v>15</v>
+      </c>
+      <c r="B150">
+        <v>9</v>
+      </c>
+      <c r="C150">
+        <v>14083158</v>
+      </c>
+      <c r="D150" t="s">
+        <v>67</v>
+      </c>
+      <c r="E150" t="s">
+        <v>79</v>
+      </c>
+      <c r="F150" t="s">
+        <v>93</v>
+      </c>
+      <c r="G150" t="s">
+        <v>89</v>
+      </c>
+      <c r="H150" t="s">
+        <v>109</v>
+      </c>
+      <c r="I150" t="s">
+        <v>138</v>
+      </c>
+      <c r="J150">
+        <v>84744</v>
+      </c>
+      <c r="K150">
+        <v>40.453</v>
+      </c>
+      <c r="L150">
+        <v>-3.6883</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12">
+      <c r="A151">
+        <v>15</v>
+      </c>
+      <c r="B151">
+        <v>10</v>
+      </c>
+      <c r="C151">
+        <v>14083160</v>
+      </c>
+      <c r="D151" t="s">
+        <v>68</v>
+      </c>
+      <c r="E151" t="s">
+        <v>79</v>
+      </c>
+      <c r="F151" t="s">
+        <v>97</v>
+      </c>
+      <c r="G151" t="s">
+        <v>96</v>
+      </c>
+      <c r="H151" t="s">
+        <v>105</v>
+      </c>
+      <c r="I151" t="s">
+        <v>142</v>
+      </c>
+      <c r="J151">
+        <v>23576</v>
+      </c>
+      <c r="K151">
+        <v>42.796662</v>
+      </c>
+      <c r="L151">
+        <v>-1.637131</v>
+      </c>
+    </row>
+    <row r="152" spans="1:12">
+      <c r="A152">
+        <v>16</v>
+      </c>
+      <c r="B152">
+        <v>1</v>
+      </c>
+      <c r="C152">
+        <v>14083177</v>
+      </c>
+      <c r="D152" t="s">
+        <v>69</v>
+      </c>
+      <c r="E152" t="s">
+        <v>79</v>
+      </c>
+      <c r="F152" t="s">
+        <v>98</v>
+      </c>
+      <c r="G152" t="s">
+        <v>84</v>
+      </c>
+      <c r="H152" t="s">
+        <v>115</v>
+      </c>
+      <c r="I152" t="s">
+        <v>143</v>
+      </c>
+      <c r="J152">
+        <v>40000</v>
+      </c>
+      <c r="K152">
+        <v>43.301337</v>
+      </c>
+      <c r="L152">
+        <v>-1.973552</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12">
+      <c r="A153">
+        <v>16</v>
+      </c>
+      <c r="B153">
+        <v>2</v>
+      </c>
+      <c r="C153">
+        <v>14083165</v>
+      </c>
+      <c r="D153" t="s">
+        <v>70</v>
+      </c>
+      <c r="E153" t="s">
+        <v>80</v>
+      </c>
+      <c r="F153" t="s">
+        <v>95</v>
+      </c>
+      <c r="G153" t="s">
+        <v>88</v>
+      </c>
+      <c r="H153" t="s">
+        <v>107</v>
+      </c>
+      <c r="I153" t="s">
+        <v>140</v>
+      </c>
+      <c r="J153">
+        <v>70460</v>
+      </c>
+      <c r="K153">
+        <v>40.436053</v>
+      </c>
+      <c r="L153">
+        <v>-3.599716</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12">
+      <c r="A154">
+        <v>16</v>
+      </c>
+      <c r="B154">
+        <v>3</v>
+      </c>
+      <c r="C154">
+        <v>14083174</v>
+      </c>
+      <c r="D154" t="s">
+        <v>70</v>
+      </c>
+      <c r="E154" t="s">
+        <v>81</v>
+      </c>
+      <c r="F154" t="s">
+        <v>86</v>
+      </c>
+      <c r="G154" t="s">
+        <v>92</v>
+      </c>
+      <c r="H154" t="s">
+        <v>119</v>
+      </c>
+      <c r="I154" t="s">
+        <v>131</v>
+      </c>
+      <c r="J154">
+        <v>26020</v>
+      </c>
+      <c r="K154">
+        <v>39.589935</v>
+      </c>
+      <c r="L154">
+        <v>2.630116</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12">
+      <c r="A155">
+        <v>16</v>
+      </c>
+      <c r="B155">
+        <v>4</v>
+      </c>
+      <c r="C155">
+        <v>14083168</v>
+      </c>
+      <c r="D155" t="s">
+        <v>70</v>
+      </c>
+      <c r="E155" t="s">
+        <v>82</v>
+      </c>
+      <c r="F155" t="s">
+        <v>103</v>
+      </c>
+      <c r="G155" t="s">
+        <v>97</v>
+      </c>
+      <c r="H155" t="s">
+        <v>105</v>
+      </c>
+      <c r="I155" t="s">
+        <v>151</v>
+      </c>
+      <c r="J155">
+        <v>45401</v>
+      </c>
+      <c r="K155">
+        <v>41.380881</v>
+      </c>
+      <c r="L155">
+        <v>2.122818</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12">
+      <c r="A156">
+        <v>16</v>
+      </c>
+      <c r="B156">
+        <v>5</v>
+      </c>
+      <c r="C156">
+        <v>14083175</v>
+      </c>
+      <c r="D156" t="s">
+        <v>70</v>
+      </c>
+      <c r="E156" t="s">
+        <v>79</v>
+      </c>
+      <c r="F156" t="s">
+        <v>102</v>
+      </c>
+      <c r="G156" t="s">
+        <v>91</v>
+      </c>
+      <c r="H156" t="s">
+        <v>117</v>
+      </c>
+      <c r="I156" t="s">
+        <v>147</v>
+      </c>
+      <c r="J156">
+        <v>17393</v>
+      </c>
+      <c r="K156">
+        <v>40.325725</v>
+      </c>
+      <c r="L156">
+        <v>-3.714933</v>
+      </c>
+    </row>
+    <row r="157" spans="1:12">
+      <c r="A157">
+        <v>16</v>
+      </c>
+      <c r="B157">
+        <v>6</v>
+      </c>
+      <c r="C157">
+        <v>14083179</v>
+      </c>
+      <c r="D157" t="s">
+        <v>71</v>
+      </c>
+      <c r="E157" t="s">
+        <v>80</v>
+      </c>
+      <c r="F157" t="s">
+        <v>100</v>
+      </c>
+      <c r="G157" t="s">
+        <v>99</v>
+      </c>
+      <c r="H157" t="s">
+        <v>126</v>
+      </c>
+      <c r="I157" t="s">
+        <v>145</v>
+      </c>
+      <c r="J157">
+        <v>42714</v>
+      </c>
+      <c r="K157">
+        <v>37.384634</v>
+      </c>
+      <c r="L157">
+        <v>-5.971156</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12">
+      <c r="A158">
+        <v>16</v>
+      </c>
+      <c r="B158">
+        <v>7</v>
+      </c>
+      <c r="C158">
+        <v>14083171</v>
+      </c>
+      <c r="D158" t="s">
+        <v>71</v>
+      </c>
+      <c r="E158" t="s">
+        <v>81</v>
+      </c>
+      <c r="F158" t="s">
+        <v>89</v>
+      </c>
+      <c r="G158" t="s">
+        <v>90</v>
+      </c>
+      <c r="H158" t="s">
+        <v>105</v>
+      </c>
+      <c r="I158" t="s">
+        <v>134</v>
+      </c>
+      <c r="J158">
+        <v>24870</v>
+      </c>
+      <c r="K158">
+        <v>42.211122</v>
+      </c>
+      <c r="L158">
+        <v>-8.739231</v>
+      </c>
+    </row>
+    <row r="159" spans="1:12">
+      <c r="A159">
+        <v>16</v>
+      </c>
+      <c r="B159">
+        <v>9</v>
+      </c>
+      <c r="C159">
+        <v>14083164</v>
+      </c>
+      <c r="D159" t="s">
+        <v>71</v>
+      </c>
+      <c r="E159" t="s">
+        <v>79</v>
+      </c>
+      <c r="F159" t="s">
+        <v>87</v>
+      </c>
+      <c r="G159" t="s">
+        <v>93</v>
+      </c>
+      <c r="H159" t="s">
+        <v>115</v>
+      </c>
+      <c r="I159" t="s">
+        <v>132</v>
+      </c>
+      <c r="J159">
+        <v>19840</v>
+      </c>
+      <c r="K159">
+        <v>42.8371</v>
+      </c>
+      <c r="L159">
+        <v>-2.6882</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12">
+      <c r="A160">
+        <v>16</v>
+      </c>
+      <c r="B160">
+        <v>10</v>
+      </c>
+      <c r="C160">
+        <v>14083173</v>
+      </c>
+      <c r="D160" t="s">
+        <v>72</v>
+      </c>
+      <c r="E160" t="s">
+        <v>79</v>
+      </c>
+      <c r="F160" t="s">
+        <v>101</v>
+      </c>
+      <c r="G160" t="s">
+        <v>94</v>
+      </c>
+      <c r="H160" t="s">
+        <v>122</v>
+      </c>
+      <c r="I160" t="s">
+        <v>146</v>
+      </c>
+      <c r="J160">
+        <v>14708</v>
+      </c>
+      <c r="K160">
+        <v>40.3921</v>
+      </c>
+      <c r="L160">
+        <v>-3.6587</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12">
+      <c r="A161">
+        <v>17</v>
+      </c>
+      <c r="B161">
+        <v>1</v>
+      </c>
+      <c r="C161">
+        <v>14083193</v>
+      </c>
+      <c r="D161" t="s">
+        <v>73</v>
+      </c>
+      <c r="E161" t="s">
+        <v>79</v>
+      </c>
+      <c r="F161" t="s">
+        <v>88</v>
+      </c>
+      <c r="G161" t="s">
+        <v>86</v>
+      </c>
+      <c r="H161" t="s">
+        <v>108</v>
+      </c>
+      <c r="I161" t="s">
+        <v>133</v>
+      </c>
+      <c r="J161">
+        <v>49430</v>
+      </c>
+      <c r="K161">
+        <v>39.474528</v>
+      </c>
+      <c r="L161">
+        <v>-0.358157</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12">
+      <c r="A162">
+        <v>17</v>
+      </c>
+      <c r="B162">
+        <v>2</v>
+      </c>
+      <c r="C162">
+        <v>14083192</v>
+      </c>
+      <c r="D162" t="s">
+        <v>74</v>
+      </c>
+      <c r="E162" t="s">
+        <v>80</v>
+      </c>
+      <c r="F162" t="s">
+        <v>99</v>
+      </c>
+      <c r="G162" t="s">
+        <v>89</v>
+      </c>
+      <c r="H162" t="s">
+        <v>122</v>
+      </c>
+      <c r="I162" t="s">
+        <v>144</v>
+      </c>
+      <c r="J162">
+        <v>30500</v>
+      </c>
+      <c r="K162">
+        <v>43.360872</v>
+      </c>
+      <c r="L162">
+        <v>-5.870332</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12">
+      <c r="A163">
+        <v>17</v>
+      </c>
+      <c r="B163">
+        <v>3</v>
+      </c>
+      <c r="C163">
+        <v>14083184</v>
+      </c>
+      <c r="D163" t="s">
+        <v>74</v>
+      </c>
+      <c r="E163" t="s">
+        <v>81</v>
+      </c>
+      <c r="F163" t="s">
+        <v>96</v>
+      </c>
+      <c r="G163" t="s">
+        <v>98</v>
+      </c>
+      <c r="H163" t="s">
+        <v>108</v>
+      </c>
+      <c r="I163" t="s">
+        <v>141</v>
+      </c>
+      <c r="J163">
+        <v>26354</v>
+      </c>
+      <c r="K163">
+        <v>39.4946</v>
+      </c>
+      <c r="L163">
+        <v>-0.3633</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12">
+      <c r="A164">
+        <v>17</v>
+      </c>
+      <c r="B164">
+        <v>4</v>
+      </c>
+      <c r="C164">
+        <v>14083188</v>
+      </c>
+      <c r="D164" t="s">
+        <v>74</v>
+      </c>
+      <c r="E164" t="s">
+        <v>82</v>
+      </c>
+      <c r="F164" t="s">
+        <v>97</v>
+      </c>
+      <c r="G164" t="s">
+        <v>87</v>
+      </c>
+      <c r="H164" t="s">
+        <v>116</v>
+      </c>
+      <c r="I164" t="s">
+        <v>142</v>
+      </c>
+      <c r="J164">
+        <v>23576</v>
+      </c>
+      <c r="K164">
+        <v>42.796662</v>
+      </c>
+      <c r="L164">
+        <v>-1.637131</v>
+      </c>
+    </row>
+    <row r="165" spans="1:12">
+      <c r="A165">
+        <v>17</v>
+      </c>
+      <c r="B165">
+        <v>5</v>
+      </c>
+      <c r="C165">
+        <v>14083185</v>
+      </c>
+      <c r="D165" t="s">
+        <v>74</v>
+      </c>
+      <c r="E165" t="s">
+        <v>79</v>
+      </c>
+      <c r="F165" t="s">
+        <v>93</v>
+      </c>
+      <c r="G165" t="s">
+        <v>100</v>
+      </c>
+      <c r="H165" t="s">
+        <v>105</v>
+      </c>
+      <c r="I165" t="s">
+        <v>138</v>
+      </c>
+      <c r="J165">
+        <v>84744</v>
+      </c>
+      <c r="K165">
+        <v>40.453</v>
+      </c>
+      <c r="L165">
+        <v>-3.6883</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implemented panel settings control
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/Server/files_initted/partidos_info.xlsx
+++ b/webscrapping/sofascore/Server/files_initted/partidos_info.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="60">
   <si>
     <t>Jornada</t>
   </si>
@@ -64,6 +64,9 @@
     <t>21/12/2025</t>
   </si>
   <si>
+    <t>22/12/2025</t>
+  </si>
+  <si>
     <t>21:00</t>
   </si>
   <si>
@@ -103,6 +106,9 @@
     <t>Real Betis</t>
   </si>
   <si>
+    <t>Athletic Club</t>
+  </si>
+  <si>
     <t>Mallorca</t>
   </si>
   <si>
@@ -130,6 +136,9 @@
     <t>Getafe</t>
   </si>
   <si>
+    <t>Espanyol</t>
+  </si>
+  <si>
     <t>1-1</t>
   </si>
   <si>
@@ -151,6 +160,9 @@
     <t>4-0</t>
   </si>
   <si>
+    <t>1-2</t>
+  </si>
+  <si>
     <t>Mestalla</t>
   </si>
   <si>
@@ -176,6 +188,9 @@
   </si>
   <si>
     <t>Estadio de la Cartuja</t>
+  </si>
+  <si>
+    <t>San Mamés</t>
   </si>
   <si>
     <t>Jornada 17</t>
@@ -536,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -594,19 +609,19 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J2">
         <v>49430</v>
@@ -618,7 +633,7 @@
         <v>-0.358157</v>
       </c>
       <c r="M2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -635,19 +650,19 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J3">
         <v>30500</v>
@@ -659,7 +674,7 @@
         <v>-5.870332</v>
       </c>
       <c r="M3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -676,19 +691,19 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="J4">
         <v>26354</v>
@@ -700,7 +715,7 @@
         <v>-0.3633</v>
       </c>
       <c r="M4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -717,19 +732,19 @@
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="J5">
         <v>23576</v>
@@ -741,7 +756,7 @@
         <v>-1.637131</v>
       </c>
       <c r="M5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -758,19 +773,19 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H6" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="J6">
         <v>84744</v>
@@ -782,7 +797,7 @@
         <v>-3.6883</v>
       </c>
       <c r="M6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -799,19 +814,19 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="J7">
         <v>14624</v>
@@ -823,7 +838,7 @@
         <v>2.8278</v>
       </c>
       <c r="M7" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -840,19 +855,19 @@
         <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J8">
         <v>23500</v>
@@ -864,7 +879,7 @@
         <v>-0.103405</v>
       </c>
       <c r="M8" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -881,19 +896,19 @@
         <v>15</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J9">
         <v>31388</v>
@@ -905,7 +920,7 @@
         <v>-0.663305</v>
       </c>
       <c r="M9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -922,19 +937,19 @@
         <v>15</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H10" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I10" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J10">
         <v>70000</v>
@@ -946,7 +961,48 @@
         <v>-6.004613</v>
       </c>
       <c r="M10" t="s">
-        <v>54</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11">
+        <v>17</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>14083180</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H11" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11">
+        <v>53289</v>
+      </c>
+      <c r="K11">
+        <v>43.264204</v>
+      </c>
+      <c r="L11">
+        <v>-2.949391</v>
+      </c>
+      <c r="M11" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
completed scrapping and settings
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/Server/files_initted/partidos_info.xlsx
+++ b/webscrapping/sofascore/Server/files_initted/partidos_info.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="48">
   <si>
     <t>Jornada</t>
   </si>
@@ -55,16 +55,13 @@
     <t>__sheet</t>
   </si>
   <si>
-    <t>19/12/2025</t>
-  </si>
-  <si>
-    <t>20/12/2025</t>
-  </si>
-  <si>
-    <t>21/12/2025</t>
-  </si>
-  <si>
-    <t>22/12/2025</t>
+    <t>12/12/2025</t>
+  </si>
+  <si>
+    <t>13/12/2025</t>
+  </si>
+  <si>
+    <t>14/12/2025</t>
   </si>
   <si>
     <t>21:00</t>
@@ -79,121 +76,88 @@
     <t>18:30</t>
   </si>
   <si>
+    <t>Real Sociedad</t>
+  </si>
+  <si>
+    <t>Atlético Madrid</t>
+  </si>
+  <si>
+    <t>Mallorca</t>
+  </si>
+  <si>
+    <t>Barcelona</t>
+  </si>
+  <si>
+    <t>Getafe</t>
+  </si>
+  <si>
+    <t>Sevilla</t>
+  </si>
+  <si>
+    <t>Celta Vigo</t>
+  </si>
+  <si>
+    <t>Girona FC</t>
+  </si>
+  <si>
     <t>Valencia</t>
   </si>
   <si>
+    <t>Elche</t>
+  </si>
+  <si>
+    <t>Osasuna</t>
+  </si>
+  <si>
+    <t>Espanyol</t>
+  </si>
+  <si>
     <t>Real Oviedo</t>
   </si>
   <si>
-    <t>Levante UD</t>
-  </si>
-  <si>
-    <t>Osasuna</t>
-  </si>
-  <si>
-    <t>Real Madrid</t>
-  </si>
-  <si>
-    <t>Girona FC</t>
-  </si>
-  <si>
-    <t>Villarreal</t>
-  </si>
-  <si>
-    <t>Elche</t>
-  </si>
-  <si>
-    <t>Real Betis</t>
-  </si>
-  <si>
     <t>Athletic Club</t>
   </si>
   <si>
-    <t>Mallorca</t>
-  </si>
-  <si>
-    <t>Celta Vigo</t>
-  </si>
-  <si>
-    <t>Real Sociedad</t>
-  </si>
-  <si>
-    <t>Deportivo Alavés</t>
-  </si>
-  <si>
-    <t>Sevilla</t>
-  </si>
-  <si>
-    <t>Atlético Madrid</t>
-  </si>
-  <si>
-    <t>Barcelona</t>
-  </si>
-  <si>
-    <t>Rayo Vallecano</t>
-  </si>
-  <si>
-    <t>Getafe</t>
-  </si>
-  <si>
-    <t>Espanyol</t>
-  </si>
-  <si>
-    <t>1-1</t>
-  </si>
-  <si>
-    <t>0-0</t>
-  </si>
-  <si>
-    <t>3-0</t>
+    <t>1-2</t>
+  </si>
+  <si>
+    <t>2-1</t>
+  </si>
+  <si>
+    <t>3-1</t>
   </si>
   <si>
     <t>2-0</t>
   </si>
   <si>
-    <t>0-3</t>
-  </si>
-  <si>
-    <t>0-2</t>
+    <t>0-1</t>
   </si>
   <si>
     <t>4-0</t>
   </si>
   <si>
-    <t>1-2</t>
-  </si>
-  <si>
-    <t>Mestalla</t>
-  </si>
-  <si>
-    <t>Carlos Tartiere</t>
-  </si>
-  <si>
-    <t>Ciudad de Valencia</t>
-  </si>
-  <si>
-    <t>Estadio El Sadar</t>
-  </si>
-  <si>
-    <t>Bernabéu</t>
-  </si>
-  <si>
-    <t>Estadi Montilivi</t>
-  </si>
-  <si>
-    <t>Estadio de la Ceramica</t>
-  </si>
-  <si>
-    <t>Estadio Martínez Valero</t>
-  </si>
-  <si>
-    <t>Estadio de la Cartuja</t>
-  </si>
-  <si>
-    <t>San Mamés</t>
-  </si>
-  <si>
-    <t>Jornada 17</t>
+    <t>Reale Arena</t>
+  </si>
+  <si>
+    <t>Riyadh Air Metropolitano</t>
+  </si>
+  <si>
+    <t>Estadi de Son Moix</t>
+  </si>
+  <si>
+    <t>Spotify Camp Nou</t>
+  </si>
+  <si>
+    <t>Coliseum Alfonso Pérez</t>
+  </si>
+  <si>
+    <t>Ramón Sánchez Pizjuán</t>
+  </si>
+  <si>
+    <t>Estadio Abanca Balaídos</t>
+  </si>
+  <si>
+    <t>Jornada 16</t>
   </si>
 </sst>
 </file>
@@ -551,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -597,412 +561,289 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2">
-        <v>14083193</v>
+        <v>14083177</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="I2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="J2">
-        <v>49430</v>
+        <v>40000</v>
       </c>
       <c r="K2">
-        <v>39.474528</v>
+        <v>43.301337</v>
       </c>
       <c r="L2">
-        <v>-0.358157</v>
+        <v>-1.973552</v>
       </c>
       <c r="M2" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3">
-        <v>14083192</v>
+        <v>14083165</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H3" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I3" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J3">
-        <v>30500</v>
+        <v>70460</v>
       </c>
       <c r="K3">
-        <v>43.360872</v>
+        <v>40.436053</v>
       </c>
       <c r="L3">
-        <v>-5.870332</v>
+        <v>-3.599716</v>
       </c>
       <c r="M3" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4">
-        <v>14083184</v>
+        <v>14083174</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="J4">
-        <v>26354</v>
+        <v>26020</v>
       </c>
       <c r="K4">
-        <v>39.4946</v>
+        <v>39.589935</v>
       </c>
       <c r="L4">
-        <v>-0.3633</v>
+        <v>2.630116</v>
       </c>
       <c r="M4" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5">
-        <v>14083188</v>
+        <v>14083168</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
         <v>43</v>
       </c>
-      <c r="I5" t="s">
-        <v>52</v>
-      </c>
       <c r="J5">
-        <v>23576</v>
+        <v>45401</v>
       </c>
       <c r="K5">
-        <v>42.796662</v>
+        <v>41.380881</v>
       </c>
       <c r="L5">
-        <v>-1.637131</v>
+        <v>2.122818</v>
       </c>
       <c r="M5" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6">
-        <v>14083185</v>
+        <v>14083175</v>
       </c>
       <c r="D6" t="s">
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" t="s">
         <v>44</v>
       </c>
-      <c r="I6" t="s">
-        <v>53</v>
-      </c>
       <c r="J6">
-        <v>84744</v>
+        <v>17393</v>
       </c>
       <c r="K6">
-        <v>40.453</v>
+        <v>40.325725</v>
       </c>
       <c r="L6">
-        <v>-3.6883</v>
+        <v>-3.714933</v>
       </c>
       <c r="M6" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7">
-        <v>14083189</v>
+        <v>14083179</v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
         <v>45</v>
       </c>
-      <c r="I7" t="s">
-        <v>54</v>
-      </c>
       <c r="J7">
-        <v>14624</v>
+        <v>42714</v>
       </c>
       <c r="K7">
-        <v>41.9611</v>
+        <v>37.384634</v>
       </c>
       <c r="L7">
-        <v>2.8278</v>
+        <v>-5.971156</v>
       </c>
       <c r="M7" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
       <c r="C8">
-        <v>14083190</v>
+        <v>14083171</v>
       </c>
       <c r="D8" t="s">
         <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" t="s">
         <v>37</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>46</v>
       </c>
-      <c r="I8" t="s">
-        <v>55</v>
-      </c>
       <c r="J8">
-        <v>23500</v>
+        <v>24870</v>
       </c>
       <c r="K8">
-        <v>39.944208</v>
+        <v>42.211122</v>
       </c>
       <c r="L8">
-        <v>-0.103405</v>
+        <v>-8.739231</v>
       </c>
       <c r="M8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9">
-        <v>17</v>
-      </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9">
-        <v>14083183</v>
-      </c>
-      <c r="D9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" t="s">
-        <v>28</v>
-      </c>
-      <c r="G9" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9" t="s">
         <v>47</v>
-      </c>
-      <c r="I9" t="s">
-        <v>56</v>
-      </c>
-      <c r="J9">
-        <v>31388</v>
-      </c>
-      <c r="K9">
-        <v>38.267044</v>
-      </c>
-      <c r="L9">
-        <v>-0.663305</v>
-      </c>
-      <c r="M9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10">
-        <v>17</v>
-      </c>
-      <c r="B10">
-        <v>9</v>
-      </c>
-      <c r="C10">
-        <v>14083181</v>
-      </c>
-      <c r="D10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" t="s">
-        <v>39</v>
-      </c>
-      <c r="H10" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" t="s">
-        <v>57</v>
-      </c>
-      <c r="J10">
-        <v>70000</v>
-      </c>
-      <c r="K10">
-        <v>37.417235</v>
-      </c>
-      <c r="L10">
-        <v>-6.004613</v>
-      </c>
-      <c r="M10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11">
-        <v>17</v>
-      </c>
-      <c r="B11">
-        <v>10</v>
-      </c>
-      <c r="C11">
-        <v>14083180</v>
-      </c>
-      <c r="D11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" t="s">
-        <v>58</v>
-      </c>
-      <c r="J11">
-        <v>53289</v>
-      </c>
-      <c r="K11">
-        <v>43.264204</v>
-      </c>
-      <c r="L11">
-        <v>-2.949391</v>
-      </c>
-      <c r="M11" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>